<commit_message>
Fixed CI headless execution
</commit_message>
<xml_diff>
--- a/test-data/createdUsers.xlsx
+++ b/test-data/createdUsers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,9 +511,23 @@
         <v>2026-05-21T10:33:43.587Z</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>user_1779792293932</v>
+      </c>
+      <c r="B9" t="str">
+        <v>user_1779792293932@mail.com</v>
+      </c>
+      <c r="C9" t="str">
+        <v>user_1779792293932_123456</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-05-26T10:44:59.741Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>